<commit_message>
Add OPP CPP costing and size-aware quotes
</commit_message>
<xml_diff>
--- a/Slider bag/报价计算方式.xlsx
+++ b/Slider bag/报价计算方式.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ai项目\世科报价系统\Slider bag\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B437949-6AB1-4DCB-A175-3F9AEA0A9F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCFAB1DB-988A-4CD7-A6A8-BFEBD02CE48C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -493,6 +493,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -518,18 +530,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -813,26 +813,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="22"/>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
+      <c r="A2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:8" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
     </row>
     <row r="4" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
@@ -931,12 +931,12 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="1:8" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
@@ -955,86 +955,86 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="21.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:8" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="23"/>
-      <c r="C13" s="26">
+      <c r="B13" s="27"/>
+      <c r="C13" s="17">
         <v>0.02</v>
       </c>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B14" s="27"/>
+      <c r="B14" s="18"/>
       <c r="C14" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D14" s="3">
         <v>100</v>
       </c>
-      <c r="E14" s="24">
+      <c r="E14" s="15">
         <v>0.98</v>
       </c>
       <c r="F14" s="10"/>
       <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="27"/>
-      <c r="B15" s="27"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="13" t="s">
         <v>24</v>
       </c>
       <c r="D15" s="3">
         <v>20</v>
       </c>
-      <c r="E15" s="25"/>
+      <c r="E15" s="16"/>
       <c r="F15" s="10"/>
       <c r="G15" s="9"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="27"/>
-      <c r="B16" s="27"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="12" t="s">
         <v>25</v>
       </c>
       <c r="D16" s="3">
         <v>10</v>
       </c>
-      <c r="E16" s="25"/>
+      <c r="E16" s="16"/>
       <c r="F16" s="10"/>
       <c r="G16" s="9"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="27"/>
-      <c r="B17" s="27"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="18"/>
       <c r="C17" s="13" t="s">
         <v>26</v>
       </c>
       <c r="D17" s="3">
         <v>5</v>
       </c>
-      <c r="E17" s="25"/>
+      <c r="E17" s="16"/>
       <c r="F17" s="10"/>
       <c r="G17" s="9"/>
     </row>
     <row r="18" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="20"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="24"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
@@ -1158,11 +1158,11 @@
       </c>
     </row>
     <row r="31" spans="1:7" ht="17.649999999999999" x14ac:dyDescent="0.3">
-      <c r="A31" s="18" t="s">
+      <c r="A31" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="B31" s="19"/>
-      <c r="C31" s="20"/>
+      <c r="B31" s="23"/>
+      <c r="C31" s="24"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
@@ -1330,16 +1330,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A1:D2"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A13:B13"/>
     <mergeCell ref="E14:E17"/>
     <mergeCell ref="C13:E13"/>
     <mergeCell ref="A14:B17"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A1:D2"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A13:B13"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="4">

</xml_diff>